<commit_message>
Fix competitiion results template
</commit_message>
<xml_diff>
--- a/owlcms/src/main/resources/templates/competitionResults/CompetitionResults-A4.xlsx
+++ b/owlcms/src/main/resources/templates/competitionResults/CompetitionResults-A4.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lamyj\git\owlcms4\owlcms\src\main\resources\templates\competitionResults\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8136B1B5-275B-4A16-9F0E-B9B4585C71ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{562B2A39-D291-400B-B415-CE5DE6964768}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-27135" yWindow="4245" windowWidth="24615" windowHeight="11310" xr2:uid="{A0CDC2EC-0CF4-1C49-B0F5-6174D88CD55E}"/>
+    <workbookView xWindow="3120" yWindow="3375" windowWidth="24615" windowHeight="11310" xr2:uid="{A0CDC2EC-0CF4-1C49-B0F5-6174D88CD55E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -446,18 +446,12 @@
     <t>${!athlete.done ? "-" : athlete.total == 0 ? "DNF" : athlete.total}</t>
   </si>
   <si>
-    <t>${!athlete.done ? "-" : athlete.total == 0 ? "DNF" : athlete.bestLifterScore}</t>
-  </si>
-  <si>
     <t>${!athlete.categoryFinished ? "-" : athlete.categoryScoreRank == 0 ? "DNF" : athlete.categoryScoreRank}</t>
   </si>
   <si>
     <t>Score</t>
   </si>
   <si>
-    <t>${!athlete.done ? "-" : athlete.total == 0 ? "DNF" : athlete.categoryScore}</t>
-  </si>
-  <si>
     <t>${group.item.category.ageGroup.scoringTitle}</t>
   </si>
   <si>
@@ -510,6 +504,12 @@
   </si>
   <si>
     <t>${group.item.category}</t>
+  </si>
+  <si>
+    <t>${!athlete.done ? "-" : athlete.total == 0 ? "-" : athlete.bestLifterScore}</t>
+  </si>
+  <si>
+    <t>${!athlete.done ? "-" : athlete.total == 0 ? "-" : athlete.categoryScore}</t>
   </si>
 </sst>
 </file>
@@ -1134,7 +1134,7 @@
     </row>
     <row r="3" spans="1:16" s="15" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B3" s="14"/>
       <c r="C3" s="14"/>
@@ -1152,46 +1152,46 @@
       <c r="E4" s="7"/>
       <c r="F4" s="7"/>
       <c r="G4" s="30" t="s">
+        <v>31</v>
+      </c>
+      <c r="H4" s="30" t="s">
+        <v>26</v>
+      </c>
+      <c r="I4" s="21" t="s">
         <v>33</v>
-      </c>
-      <c r="H4" s="30" t="s">
-        <v>28</v>
-      </c>
-      <c r="I4" s="21" t="s">
-        <v>35</v>
       </c>
       <c r="J4" s="22"/>
       <c r="K4" s="23"/>
       <c r="L4" s="21" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="M4" s="22"/>
       <c r="N4" s="23"/>
       <c r="O4" s="30" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="P4" s="28" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="D5" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="E5" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="C5" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="E5" s="8" t="s">
+      <c r="F5" s="8" t="s">
         <v>25</v>
-      </c>
-      <c r="F5" s="8" t="s">
-        <v>27</v>
       </c>
       <c r="G5" s="31"/>
       <c r="H5" s="31"/>
@@ -1218,7 +1218,7 @@
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>13</v>
@@ -1263,7 +1263,7 @@
         <v>14</v>
       </c>
       <c r="P6" s="3" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
@@ -1286,7 +1286,7 @@
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="25" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B8" s="26"/>
       <c r="C8" s="27"/>
@@ -1294,42 +1294,42 @@
       <c r="E8" s="7"/>
       <c r="F8" s="7"/>
       <c r="G8" s="30" t="s">
+        <v>24</v>
+      </c>
+      <c r="H8" s="30" t="s">
         <v>26</v>
       </c>
-      <c r="H8" s="30" t="s">
-        <v>28</v>
-      </c>
       <c r="I8" s="21" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="J8" s="22"/>
       <c r="K8" s="23"/>
       <c r="L8" s="21" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="M8" s="22"/>
       <c r="N8" s="23"/>
       <c r="O8" s="30" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="P8" s="12" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="17" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B9" s="18"/>
       <c r="C9" s="19"/>
       <c r="D9" s="8" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E9" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="F9" s="8" t="s">
         <v>25</v>
-      </c>
-      <c r="F9" s="8" t="s">
-        <v>27</v>
       </c>
       <c r="G9" s="31"/>
       <c r="H9" s="31"/>
@@ -1353,12 +1353,12 @@
       </c>
       <c r="O9" s="31"/>
       <c r="P9" s="8" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="20" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B10" s="20"/>
       <c r="C10" s="20"/>
@@ -1399,7 +1399,7 @@
         <v>14</v>
       </c>
       <c r="P10" s="3" t="s">
-        <v>18</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fixed headers and extra
</commit_message>
<xml_diff>
--- a/owlcms/src/main/resources/templates/competitionResults/CompetitionResults-A4.xlsx
+++ b/owlcms/src/main/resources/templates/competitionResults/CompetitionResults-A4.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lamyj\git\owlcms4\owlcms\src\main\resources\templates\competitionResults\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{562B2A39-D291-400B-B415-CE5DE6964768}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0A127284-201C-4DFD-924B-7D1809DE9AE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3120" yWindow="3375" windowWidth="24615" windowHeight="11310" xr2:uid="{A0CDC2EC-0CF4-1C49-B0F5-6174D88CD55E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{A0CDC2EC-0CF4-1C49-B0F5-6174D88CD55E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -399,7 +399,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="35">
   <si>
     <t>${competition.competitionName}</t>
   </si>
@@ -437,18 +437,9 @@
     <t>${athlete.cleanJerk3AsInteger == 0 ? "-" : athlete.cleanJerk3AsInteger}</t>
   </si>
   <si>
-    <t>${!athlete.categoryFinished ? "-" : athlete.cleanJerkRank == 0 ? "DNF" : athlete.cleanJerkRank}</t>
-  </si>
-  <si>
-    <t>${!athlete.categoryFinished ? "-" : athlete.snatchRank == 0 ? "DNF" : athlete.snatchRank}</t>
-  </si>
-  <si>
     <t>${!athlete.done ? "-" : athlete.total == 0 ? "DNF" : athlete.total}</t>
   </si>
   <si>
-    <t>${!athlete.categoryFinished ? "-" : athlete.categoryScoreRank == 0 ? "DNF" : athlete.categoryScoreRank}</t>
-  </si>
-  <si>
     <t>Score</t>
   </si>
   <si>
@@ -482,12 +473,6 @@
     <t>${t.get("Age")}</t>
   </si>
   <si>
-    <t>${t.get("Snatch")}</t>
-  </si>
-  <si>
-    <t>${t.get("Clean_Jerk")}</t>
-  </si>
-  <si>
     <t>${t.get("Rank")}</t>
   </si>
   <si>
@@ -497,12 +482,6 @@
     <t>${t.get("Results.BodyWeight")}</t>
   </si>
   <si>
-    <t>${t.get("Results.cleanJerk")}</t>
-  </si>
-  <si>
-    <t>${t.get("Results.snatch")}</t>
-  </si>
-  <si>
     <t>${group.item.category}</t>
   </si>
   <si>
@@ -510,6 +489,21 @@
   </si>
   <si>
     <t>${!athlete.done ? "-" : athlete.total == 0 ? "-" : athlete.categoryScore}</t>
+  </si>
+  <si>
+    <t>${!athlete.categoryFinished ? "-" : athlete.categoryScoreRank == 0 ? "DNF" : (athlete.categoryScoreRank == -1 ? t.get("Results.Extra/Invited") : athlete.categoryScoreRank)}</t>
+  </si>
+  <si>
+    <t>${!athlete.categoryFinished ? "-" : athlete.snatchRank == 0 ? "DNF" : (athlete.snatchRank == -1 ? t.get("Results.Extra/Invited") : athlete.snatchRank)}</t>
+  </si>
+  <si>
+    <t>${!athlete.categoryFinished ? "-" : athlete.cleanJerkRank == 0 ? "DNF" : (athlete.cleanJerkRank == -1 ? t.get("Results.Extra/Invited") : athlete.cleanJerkRank)}</t>
+  </si>
+  <si>
+    <t>${t.get("Results.Snatch")}</t>
+  </si>
+  <si>
+    <t>${t.get("Results.Clean_and_Jerk")}</t>
   </si>
 </sst>
 </file>
@@ -1134,7 +1128,7 @@
     </row>
     <row r="3" spans="1:16" s="15" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B3" s="14"/>
       <c r="C3" s="14"/>
@@ -1152,10 +1146,10 @@
       <c r="E4" s="7"/>
       <c r="F4" s="7"/>
       <c r="G4" s="30" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="H4" s="30" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I4" s="21" t="s">
         <v>33</v>
@@ -1163,35 +1157,35 @@
       <c r="J4" s="22"/>
       <c r="K4" s="23"/>
       <c r="L4" s="21" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="M4" s="22"/>
       <c r="N4" s="23"/>
       <c r="O4" s="30" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="P4" s="28" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="B5" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="D5" s="8" t="s">
+      <c r="F5" s="8" t="s">
         <v>22</v>
-      </c>
-      <c r="E5" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="F5" s="8" t="s">
-        <v>25</v>
       </c>
       <c r="G5" s="31"/>
       <c r="H5" s="31"/>
@@ -1218,13 +1212,13 @@
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>12</v>
+        <v>32</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>1</v>
@@ -1260,10 +1254,10 @@
         <v>11</v>
       </c>
       <c r="O6" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="P6" s="3" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
@@ -1286,7 +1280,7 @@
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="25" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B8" s="26"/>
       <c r="C8" s="27"/>
@@ -1294,42 +1288,42 @@
       <c r="E8" s="7"/>
       <c r="F8" s="7"/>
       <c r="G8" s="30" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="H8" s="30" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I8" s="21" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="J8" s="22"/>
       <c r="K8" s="23"/>
       <c r="L8" s="21" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="M8" s="22"/>
       <c r="N8" s="23"/>
       <c r="O8" s="30" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="P8" s="12" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="17" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="B9" s="18"/>
       <c r="C9" s="19"/>
       <c r="D9" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="F9" s="8" t="s">
         <v>22</v>
-      </c>
-      <c r="E9" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="F9" s="8" t="s">
-        <v>25</v>
       </c>
       <c r="G9" s="31"/>
       <c r="H9" s="31"/>
@@ -1353,12 +1347,12 @@
       </c>
       <c r="O9" s="31"/>
       <c r="P9" s="8" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="20" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B10" s="20"/>
       <c r="C10" s="20"/>
@@ -1396,10 +1390,10 @@
         <v>11</v>
       </c>
       <c r="O10" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="P10" s="3" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>